<commit_message>
Add sample inference data and output artifacts
</commit_message>
<xml_diff>
--- a/output/dataset_234.xlsx
+++ b/output/dataset_234.xlsx
@@ -481,17 +481,17 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Drop width (cm)</t>
+          <t>status</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Estimated Width (μm)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Estimated Width</t>
+          <t>Measured Width (μm)</t>
         </is>
       </c>
     </row>
@@ -528,15 +528,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
         <v>3956.60791015625</v>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -571,15 +571,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
         <v>3976.8828125</v>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -614,15 +614,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>3979.48779296875</v>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -657,15 +657,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>3971.180908203125</v>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -700,15 +700,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>3961.768798828125</v>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -743,15 +743,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
         <v>3945.6806640625</v>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -786,15 +786,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>3926.5986328125</v>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -829,15 +829,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
         <v>3905.63037109375</v>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -872,15 +872,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
         <v>3891.285400390625</v>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -915,15 +915,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
         <v>3883.034423828125</v>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -958,15 +958,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M12" t="n">
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
         <v>3879.004150390625</v>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1001,15 +1001,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M13" t="n">
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
         <v>3880.080322265625</v>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1044,15 +1044,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M14" t="n">
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
         <v>3876.373291015625</v>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1087,15 +1087,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M15" t="n">
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
         <v>3873.163330078125</v>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1130,15 +1130,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M16" t="n">
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
         <v>3873.962646484375</v>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1173,15 +1173,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
         <v>3869.127685546875</v>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1216,15 +1216,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
         <v>3866.229248046875</v>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1259,15 +1259,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
         <v>3863.684326171875</v>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1302,15 +1302,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M20" t="n">
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
         <v>3858.054931640625</v>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1345,15 +1345,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M21" t="n">
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
         <v>3857.64697265625</v>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1388,15 +1388,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
         <v>3859.42529296875</v>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1431,15 +1431,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
         <v>3864.560791015625</v>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1474,15 +1474,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M24" t="n">
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
         <v>3866.517333984375</v>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1517,15 +1517,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M25" t="n">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>3865.748291015625</v>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1560,15 +1560,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M26" t="n">
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
         <v>3856.59814453125</v>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1603,15 +1603,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M27" t="n">
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
         <v>3858.74658203125</v>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1646,15 +1646,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M28" t="n">
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
         <v>3857.341552734375</v>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1689,15 +1689,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M29" t="n">
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
         <v>3852.386962890625</v>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1732,15 +1732,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M30" t="n">
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
         <v>3844.1689453125</v>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1775,15 +1775,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
         <v>3842.4482421875</v>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1818,15 +1818,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M32" t="n">
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
         <v>3843.72802734375</v>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1861,15 +1861,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M33" t="n">
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
         <v>3846.435791015625</v>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1904,15 +1904,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M34" t="n">
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
         <v>3845.692626953125</v>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1947,15 +1947,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M35" t="n">
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
         <v>3843.548583984375</v>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1990,15 +1990,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M36" t="n">
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
         <v>3843.667236328125</v>
       </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2033,15 +2033,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M37" t="n">
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
         <v>3845.88916015625</v>
       </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2076,15 +2076,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
         <v>3845.681640625</v>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2119,15 +2119,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M39" t="n">
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
         <v>3846.474853515625</v>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2162,15 +2162,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M40" t="n">
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
         <v>3843.49560546875</v>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2205,15 +2205,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M41" t="n">
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
         <v>3839.199951171875</v>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2248,15 +2248,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M42" t="n">
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
         <v>3830.32958984375</v>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2291,15 +2291,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M43" t="n">
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
         <v>3830.077880859375</v>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2334,15 +2334,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M44" t="n">
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
         <v>3837.554931640625</v>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2377,15 +2377,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M45" t="n">
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
         <v>3843.009521484375</v>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2420,15 +2420,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
         <v>3835.750732421875</v>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2463,15 +2463,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M47" t="n">
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
         <v>3832.976806640625</v>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2506,15 +2506,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M48" t="n">
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
         <v>3837.536376953125</v>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2549,15 +2549,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
         <v>3835.1513671875</v>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2592,15 +2592,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
         <v>3835.977294921875</v>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2635,15 +2635,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
         <v>3838.025146484375</v>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2678,15 +2678,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M52" t="n">
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
         <v>3834.266845703125</v>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2721,15 +2721,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M53" t="n">
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
         <v>3832.99951171875</v>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2764,15 +2764,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M54" t="n">
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
         <v>3830.589111328125</v>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2807,15 +2807,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M55" t="n">
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
         <v>3832.80029296875</v>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2850,15 +2850,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M56" t="n">
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
         <v>3828.745361328125</v>
       </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2893,15 +2893,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M57" t="n">
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
         <v>3823.612060546875</v>
       </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2936,15 +2936,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M58" t="n">
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
         <v>3829.111083984375</v>
       </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2979,15 +2979,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M59" t="n">
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
         <v>3828.423583984375</v>
       </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3022,15 +3022,15 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
         <v>3836.55029296875</v>
       </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3065,16 +3065,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K61" t="n">
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
+        <v>3837.856201171875</v>
+      </c>
+      <c r="M61" t="n">
         <v>3792.82884178058</v>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M61" t="n">
-        <v>3837.856201171875</v>
       </c>
     </row>
     <row r="62">
@@ -3110,16 +3110,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>3851.552490234375</v>
+      </c>
+      <c r="M62" t="n">
         <v>3765.31350374309</v>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M62" t="n">
-        <v>3851.552490234375</v>
       </c>
     </row>
     <row r="63">
@@ -3155,16 +3155,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K63" t="n">
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>3846.597900390625</v>
+      </c>
+      <c r="M63" t="n">
         <v>3758.39696300535</v>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
-        <v>3846.597900390625</v>
       </c>
     </row>
     <row r="64">
@@ -3200,16 +3200,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K64" t="n">
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>3863.940185546875</v>
+      </c>
+      <c r="M64" t="n">
         <v>3762.78718644225</v>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M64" t="n">
-        <v>3863.940185546875</v>
       </c>
     </row>
     <row r="65">
@@ -3245,16 +3245,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K65" t="n">
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>3875.77001953125</v>
+      </c>
+      <c r="M65" t="n">
         <v>3775.42486521917</v>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M65" t="n">
-        <v>3875.77001953125</v>
       </c>
     </row>
     <row r="66">
@@ -3290,16 +3290,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K66" t="n">
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>3875.64697265625</v>
+      </c>
+      <c r="M66" t="n">
         <v>3782.13361006083</v>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M66" t="n">
-        <v>3875.64697265625</v>
       </c>
     </row>
     <row r="67">
@@ -3335,16 +3335,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K67" t="n">
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>3854.085205078125</v>
+      </c>
+      <c r="M67" t="n">
         <v>3763.83538665976</v>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M67" t="n">
-        <v>3854.085205078125</v>
       </c>
     </row>
     <row r="68">
@@ -3380,16 +3380,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K68" t="n">
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>3811.31591796875</v>
+      </c>
+      <c r="M68" t="n">
         <v>3783.39125273461</v>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M68" t="n">
-        <v>3811.31591796875</v>
       </c>
     </row>
     <row r="69">
@@ -3425,16 +3425,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K69" t="n">
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>3807.652099609375</v>
+      </c>
+      <c r="M69" t="n">
         <v>3822.72461188601</v>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M69" t="n">
-        <v>3807.652099609375</v>
       </c>
     </row>
     <row r="70">
@@ -3470,16 +3470,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K70" t="n">
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>3808.5361328125</v>
+      </c>
+      <c r="M70" t="n">
         <v>3838.4556832935</v>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
-        <v>3808.5361328125</v>
       </c>
     </row>
     <row r="71">
@@ -3515,16 +3515,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K71" t="n">
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>3808.769287109375</v>
+      </c>
+      <c r="M71" t="n">
         <v>3838.53093109422</v>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M71" t="n">
-        <v>3808.769287109375</v>
       </c>
     </row>
     <row r="72">
@@ -3560,16 +3560,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K72" t="n">
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>3803.2353515625</v>
+      </c>
+      <c r="M72" t="n">
         <v>3835.26794276399</v>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M72" t="n">
-        <v>3803.2353515625</v>
       </c>
     </row>
     <row r="73">
@@ -3605,16 +3605,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K73" t="n">
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>3793.427734375</v>
+      </c>
+      <c r="M73" t="n">
         <v>3842.81989107939</v>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M73" t="n">
-        <v>3793.427734375</v>
       </c>
     </row>
     <row r="74">
@@ -3650,16 +3650,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K74" t="n">
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>3757.303955078125</v>
+      </c>
+      <c r="M74" t="n">
         <v>3847.88948525104</v>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M74" t="n">
-        <v>3757.303955078125</v>
       </c>
     </row>
     <row r="75">
@@ -3695,16 +3695,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K75" t="n">
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>3725.033935546875</v>
+      </c>
+      <c r="M75" t="n">
         <v>3851.77026296488</v>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M75" t="n">
-        <v>3725.033935546875</v>
       </c>
     </row>
     <row r="76">
@@ -3740,16 +3740,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K76" t="n">
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>3720.41015625</v>
+      </c>
+      <c r="M76" t="n">
         <v>3844.09926834769</v>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M76" t="n">
-        <v>3720.41015625</v>
       </c>
     </row>
     <row r="77">
@@ -3785,16 +3785,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K77" t="n">
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>3718.702880859375</v>
+      </c>
+      <c r="M77" t="n">
         <v>3813.81293416499</v>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M77" t="n">
-        <v>3718.702880859375</v>
       </c>
     </row>
     <row r="78">
@@ -3830,16 +3830,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K78" t="n">
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>3709.541748046875</v>
+      </c>
+      <c r="M78" t="n">
         <v>3770.27640081438</v>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M78" t="n">
-        <v>3709.541748046875</v>
       </c>
     </row>
     <row r="79">
@@ -3875,16 +3875,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K79" t="n">
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>3667.004150390625</v>
+      </c>
+      <c r="M79" t="n">
         <v>3750.57102707419</v>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M79" t="n">
-        <v>3667.004150390625</v>
       </c>
     </row>
     <row r="80">
@@ -3920,16 +3920,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K80" t="n">
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>3611.57373046875</v>
+      </c>
+      <c r="M80" t="n">
         <v>3721.29238772831</v>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M80" t="n">
-        <v>3611.57373046875</v>
       </c>
     </row>
     <row r="81">
@@ -3965,16 +3965,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K81" t="n">
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>3606.55859375</v>
+      </c>
+      <c r="M81" t="n">
         <v>3739.2198057744</v>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M81" t="n">
-        <v>3606.55859375</v>
       </c>
     </row>
     <row r="82">
@@ -4010,16 +4010,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K82" t="n">
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>3694.32177734375</v>
+      </c>
+      <c r="M82" t="n">
         <v>3781.32103260663</v>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M82" t="n">
-        <v>3694.32177734375</v>
       </c>
     </row>
     <row r="83">
@@ -4055,16 +4055,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K83" t="n">
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>3886.2734375</v>
+      </c>
+      <c r="M83" t="n">
         <v>3878.74519994773</v>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M83" t="n">
-        <v>3886.2734375</v>
       </c>
     </row>
     <row r="84">
@@ -4100,16 +4100,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K84" t="n">
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>4015.550537109375</v>
+      </c>
+      <c r="M84" t="n">
         <v>4046.38807922036</v>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M84" t="n">
-        <v>4015.550537109375</v>
       </c>
     </row>
     <row r="85">
@@ -4145,16 +4145,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K85" t="n">
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>4062.996337890625</v>
+      </c>
+      <c r="M85" t="n">
         <v>4096.85267923005</v>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M85" t="n">
-        <v>4062.996337890625</v>
       </c>
     </row>
     <row r="86">
@@ -4190,16 +4190,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K86" t="n">
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>4119.9052734375</v>
+      </c>
+      <c r="M86" t="n">
         <v>4088.9508368741</v>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M86" t="n">
-        <v>4119.9052734375</v>
       </c>
     </row>
     <row r="87">
@@ -4235,16 +4235,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K87" t="n">
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>4140.77734375</v>
+      </c>
+      <c r="M87" t="n">
         <v>4070.04750260288</v>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M87" t="n">
-        <v>4140.77734375</v>
       </c>
     </row>
     <row r="88">
@@ -4280,16 +4280,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K88" t="n">
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>4140.3544921875</v>
+      </c>
+      <c r="M88" t="n">
         <v>4055.79290171854</v>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M88" t="n">
-        <v>4140.3544921875</v>
       </c>
     </row>
     <row r="89">
@@ -4325,16 +4325,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K89" t="n">
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>4111.75830078125</v>
+      </c>
+      <c r="M89" t="n">
         <v>4047.77942258164</v>
-      </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M89" t="n">
-        <v>4111.75830078125</v>
       </c>
     </row>
     <row r="90">
@@ -4370,16 +4370,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K90" t="n">
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>3972.29931640625</v>
+      </c>
+      <c r="M90" t="n">
         <v>4052.52596164384</v>
-      </c>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M90" t="n">
-        <v>3972.29931640625</v>
       </c>
     </row>
     <row r="91">
@@ -4415,16 +4415,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K91" t="n">
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>3853.699462890625</v>
+      </c>
+      <c r="M91" t="n">
         <v>4050.82621755881</v>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M91" t="n">
-        <v>3853.699462890625</v>
       </c>
     </row>
     <row r="92">
@@ -4460,16 +4460,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K92" t="n">
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>3851.015869140625</v>
+      </c>
+      <c r="M92" t="n">
         <v>4010.94504783191</v>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M92" t="n">
-        <v>3851.015869140625</v>
       </c>
     </row>
     <row r="93">
@@ -4505,16 +4505,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K93" t="n">
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>3851.07568359375</v>
+      </c>
+      <c r="M93" t="n">
         <v>3921.62936615073</v>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M93" t="n">
-        <v>3851.07568359375</v>
       </c>
     </row>
     <row r="94">
@@ -4550,16 +4550,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K94" t="n">
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>3817.84716796875</v>
+      </c>
+      <c r="M94" t="n">
         <v>3883.50112440302</v>
-      </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M94" t="n">
-        <v>3817.84716796875</v>
       </c>
     </row>
     <row r="95">
@@ -4595,16 +4595,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K95" t="n">
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>3788.816162109375</v>
+      </c>
+      <c r="M95" t="n">
         <v>3867.41686583459</v>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M95" t="n">
-        <v>3788.816162109375</v>
       </c>
     </row>
     <row r="96">
@@ -4640,16 +4640,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K96" t="n">
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>3781.75634765625</v>
+      </c>
+      <c r="M96" t="n">
         <v>3869.5348362081</v>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M96" t="n">
-        <v>3781.75634765625</v>
       </c>
     </row>
     <row r="97">
@@ -4685,16 +4685,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K97" t="n">
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
+        <v>3800.111083984375</v>
+      </c>
+      <c r="M97" t="n">
         <v>3853.11500867276</v>
-      </c>
-      <c r="L97" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M97" t="n">
-        <v>3800.111083984375</v>
       </c>
     </row>
     <row r="98">
@@ -4730,16 +4730,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K98" t="n">
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>3819.82080078125</v>
+      </c>
+      <c r="M98" t="n">
         <v>3845.57919664723</v>
-      </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M98" t="n">
-        <v>3819.82080078125</v>
       </c>
     </row>
     <row r="99">
@@ -4775,16 +4775,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K99" t="n">
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
+        <v>3819.071044921875</v>
+      </c>
+      <c r="M99" t="n">
         <v>3847.45512267269</v>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M99" t="n">
-        <v>3819.071044921875</v>
       </c>
     </row>
     <row r="100">
@@ -4820,16 +4820,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K100" t="n">
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L100" t="n">
+        <v>3794.114013671875</v>
+      </c>
+      <c r="M100" t="n">
         <v>3854.94285514064</v>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M100" t="n">
-        <v>3794.114013671875</v>
       </c>
     </row>
     <row r="101">
@@ -4865,16 +4865,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K101" t="n">
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L101" t="n">
+        <v>3755.675537109375</v>
+      </c>
+      <c r="M101" t="n">
         <v>3851.14687527662</v>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M101" t="n">
-        <v>3755.675537109375</v>
       </c>
     </row>
     <row r="102">
@@ -4910,16 +4910,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K102" t="n">
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L102" t="n">
+        <v>3760.673828125</v>
+      </c>
+      <c r="M102" t="n">
         <v>3832.79233951702</v>
-      </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M102" t="n">
-        <v>3760.673828125</v>
       </c>
     </row>
     <row r="103">
@@ -4955,16 +4955,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K103" t="n">
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L103" t="n">
+        <v>3798.799560546875</v>
+      </c>
+      <c r="M103" t="n">
         <v>3835.08204611844</v>
-      </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M103" t="n">
-        <v>3798.799560546875</v>
       </c>
     </row>
     <row r="104">
@@ -5000,16 +5000,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K104" t="n">
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L104" t="n">
+        <v>3764.74658203125</v>
+      </c>
+      <c r="M104" t="n">
         <v>3844.31562635677</v>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M104" t="n">
-        <v>3764.74658203125</v>
       </c>
     </row>
     <row r="105">
@@ -5045,16 +5045,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K105" t="n">
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
+        <v>3744.986328125</v>
+      </c>
+      <c r="M105" t="n">
         <v>3881.31893818207</v>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M105" t="n">
-        <v>3744.986328125</v>
       </c>
     </row>
     <row r="106">
@@ -5090,16 +5090,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K106" t="n">
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>3760.647216796875</v>
+      </c>
+      <c r="M106" t="n">
         <v>3945.75921177978</v>
-      </c>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M106" t="n">
-        <v>3760.647216796875</v>
       </c>
     </row>
     <row r="107">
@@ -5135,16 +5135,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K107" t="n">
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L107" t="n">
+        <v>3837.311767578125</v>
+      </c>
+      <c r="M107" t="n">
         <v>3962.08452676016</v>
-      </c>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M107" t="n">
-        <v>3837.311767578125</v>
       </c>
     </row>
     <row r="108">
@@ -5180,16 +5180,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K108" t="n">
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L108" t="n">
+        <v>3875.468994140625</v>
+      </c>
+      <c r="M108" t="n">
         <v>3962.33727374946</v>
-      </c>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M108" t="n">
-        <v>3875.468994140625</v>
       </c>
     </row>
     <row r="109">
@@ -5225,16 +5225,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K109" t="n">
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L109" t="n">
+        <v>3900.15185546875</v>
+      </c>
+      <c r="M109" t="n">
         <v>3964.84465560811</v>
-      </c>
-      <c r="L109" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M109" t="n">
-        <v>3900.15185546875</v>
       </c>
     </row>
     <row r="110">
@@ -5270,16 +5270,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K110" t="n">
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L110" t="n">
+        <v>3924.033203125</v>
+      </c>
+      <c r="M110" t="n">
         <v>3971.01991494792</v>
-      </c>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M110" t="n">
-        <v>3924.033203125</v>
       </c>
     </row>
     <row r="111">
@@ -5315,16 +5315,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K111" t="n">
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>3918.498046875</v>
+      </c>
+      <c r="M111" t="n">
         <v>3965.72737652643</v>
-      </c>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M111" t="n">
-        <v>3918.498046875</v>
       </c>
     </row>
     <row r="112">
@@ -5360,16 +5360,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K112" t="n">
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>3941.31396484375</v>
+      </c>
+      <c r="M112" t="n">
         <v>3940.15234501785</v>
-      </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M112" t="n">
-        <v>3941.31396484375</v>
       </c>
     </row>
     <row r="113">
@@ -5405,16 +5405,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K113" t="n">
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>3953.334716796875</v>
+      </c>
+      <c r="M113" t="n">
         <v>3923.24875809844</v>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M113" t="n">
-        <v>3953.334716796875</v>
       </c>
     </row>
     <row r="114">
@@ -5450,16 +5450,16 @@
           <t>800by3000by23</t>
         </is>
       </c>
-      <c r="K114" t="n">
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>final validation</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>3918.106689453125</v>
+      </c>
+      <c r="M114" t="n">
         <v>3923.05446399592</v>
-      </c>
-      <c r="L114" t="inlineStr">
-        <is>
-          <t>final validation</t>
-        </is>
-      </c>
-      <c r="M114" t="n">
-        <v>3918.106689453125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>